<commit_message>
Timetable update and cleaning
Deleted keep alive workflow and added Room Numbers for every class
</commit_message>
<xml_diff>
--- a/Timetable automate.xlsx
+++ b/Timetable automate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\GitHub\TimeTable-Notifier\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3407E790-D425-4648-A963-953F5919E9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDFE58D0-D17A-4CEB-B543-00115D5F040B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{14E72CCB-0E79-4B7E-BD78-A2B34D426CDB}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{14E72CCB-0E79-4B7E-BD78-A2B34D426CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -72,21 +72,6 @@
     <t>S4</t>
   </si>
   <si>
-    <t>Web Frameworks (3:50-5:10)</t>
-  </si>
-  <si>
-    <t>OS (2:30-3:50)</t>
-  </si>
-  <si>
-    <t>IS (9:50-11:10)</t>
-  </si>
-  <si>
-    <t>IS (11:10-12:30)</t>
-  </si>
-  <si>
-    <t>AOA 92:30-3:50) R10</t>
-  </si>
-  <si>
     <t>Fehm ul Quran (11:10-12:30) R13</t>
   </si>
   <si>
@@ -118,6 +103,21 @@
   </si>
   <si>
     <t>AOA (3:50-5:10) R11</t>
+  </si>
+  <si>
+    <t>AOA (2:30-3:50) R10</t>
+  </si>
+  <si>
+    <t>Web Frameworks (3:50-5:10) L2</t>
+  </si>
+  <si>
+    <t>OS (2:30-3:50) L3</t>
+  </si>
+  <si>
+    <t>IS (9:50-11:10) L2</t>
+  </si>
+  <si>
+    <t>IS (11:10-12:30) L2</t>
   </si>
 </sst>
 </file>
@@ -534,16 +534,16 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -551,16 +551,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -568,16 +568,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -585,16 +585,16 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changed workflow time and timetable
changed worksflow time to 7:21 pm and change timetable as per new timetable
</commit_message>
<xml_diff>
--- a/Timetable automate.xlsx
+++ b/Timetable automate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\GitHub\TimeTable-Notifier\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36143FEA-9F77-4973-96C0-0F7C4B5EB2AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97860BF-7275-4201-B7B3-BF7398AC4BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{14E72CCB-0E79-4B7E-BD78-A2B34D426CDB}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{14E72CCB-0E79-4B7E-BD78-A2B34D426CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -102,9 +102,6 @@
     <t>COAL ( 2:30-3:50) L2</t>
   </si>
   <si>
-    <t>AOA (3:50-5:10) R11</t>
-  </si>
-  <si>
     <t>AOA (2:30-3:50) R10</t>
   </si>
   <si>
@@ -121,6 +118,9 @@
   </si>
   <si>
     <t>S5</t>
+  </si>
+  <si>
+    <t>AOA (9:50 - 11:10 )</t>
   </si>
 </sst>
 </file>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="I1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -540,6 +540,9 @@
       <c r="A3" t="s">
         <v>0</v>
       </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
@@ -550,7 +553,7 @@
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -567,7 +570,7 @@
         <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -578,13 +581,13 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -599,9 +602,6 @@
       </c>
       <c r="F6" t="s">
         <v>24</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>